<commit_message>
3mb swap variable validacion
</commit_message>
<xml_diff>
--- a/data/validacion_variable/elmo_data.xlsx
+++ b/data/validacion_variable/elmo_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TECNO-MASTER\Desktop\Elmo_infrastructure_sizing_NP-\data\validacion_variable\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B11E92E3-EC43-42A6-A4EA-4F9AF3CBE658}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE4E6592-5040-4FBB-8DB8-B7E3A771BA49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1860" yWindow="1860" windowWidth="21600" windowHeight="11295" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Batteries" sheetId="1" r:id="rId1"/>

</xml_diff>